<commit_message>
Update CdaTEL to ContactPoint mappings and descriptions 59aaf049f4add2dc9e338d83416583123ea92df2
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaTELToContactPointConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaTELToContactPointConceptMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaTELToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaTELToContactPointConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T14:05:46+00:00</t>
+    <t>2026-07-22T14:07:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -123,22 +123,40 @@
     <t>ContactPoint.value</t>
   </si>
   <si>
+    <t>The actual contact point details</t>
+  </si>
+  <si>
     <t>ContactPoint.system</t>
   </si>
   <si>
+    <t>phone | fax | email | pager | url | sms | other</t>
+  </si>
+  <si>
     <t>TEL.use</t>
   </si>
   <si>
+    <t>Use Code</t>
+  </si>
+  <si>
     <t>ContactPoint.use</t>
   </si>
   <si>
+    <t>home | work | temp | old | mobile - purpose of this contact point</t>
+  </si>
+  <si>
     <t>TEL.useablePeriod</t>
   </si>
   <si>
+    <t>Useable Period</t>
+  </si>
+  <si>
     <t>equivalent</t>
   </si>
   <si>
     <t>ContactPoint.period</t>
+  </si>
+  <si>
+    <t>Time period when the contact point was/is in use</t>
   </si>
 </sst>
 </file>
@@ -445,7 +463,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -459,44 +477,44 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>